<commit_message>
Absensi Agustus: sistem versi (v1.0 sumber awal kosong, rantai v-tgl-1/3/4), hapus snapshot stale, absensi.py ke versi terbaru
</commit_message>
<xml_diff>
--- a/PC-06/docs/Absensi T.P 2026-2027/ABSENSI Agustus.xlsx
+++ b/PC-06/docs/Absensi T.P 2026-2027/ABSENSI Agustus.xlsx
@@ -682,7 +682,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AO50"/>
+  <dimension ref="A1:AW99"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="14.453125" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col width="6.453125" customWidth="1" style="36" min="1" max="1"/>
@@ -1178,11 +1178,7 @@
           <t>Eireen Lorenzo</t>
         </is>
       </c>
-      <c r="D9" s="8" t="inlineStr">
-        <is>
-          <t>I</t>
-        </is>
-      </c>
+      <c r="D9" s="8" t="n"/>
       <c r="E9" s="8" t="n"/>
       <c r="F9" s="8" t="n"/>
       <c r="G9" s="8" t="n"/>
@@ -1416,16 +1412,8 @@
       </c>
       <c r="D14" s="8" t="n"/>
       <c r="E14" s="8" t="n"/>
-      <c r="F14" s="8" t="inlineStr">
-        <is>
-          <t>I</t>
-        </is>
-      </c>
-      <c r="G14" s="8" t="inlineStr">
-        <is>
-          <t>I</t>
-        </is>
-      </c>
+      <c r="F14" s="8" t="n"/>
+      <c r="G14" s="8" t="n"/>
       <c r="H14" s="8" t="n"/>
       <c r="I14" s="8" t="n"/>
       <c r="J14" s="8" t="n"/>
@@ -3906,7 +3894,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AO51"/>
+  <dimension ref="A1:AW99"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="14.453125" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col width="6.453125" customWidth="1" style="36" min="1" max="1"/>
@@ -4670,11 +4658,7 @@
       </c>
       <c r="D15" s="8" t="n"/>
       <c r="E15" s="8" t="n"/>
-      <c r="F15" s="8" t="inlineStr">
-        <is>
-          <t>S</t>
-        </is>
-      </c>
+      <c r="F15" s="8" t="n"/>
       <c r="G15" s="8" t="n"/>
       <c r="H15" s="8" t="n"/>
       <c r="I15" s="8" t="n"/>
@@ -5316,11 +5300,7 @@
           <t>Matthew Batara Hamonangan Nainggolan</t>
         </is>
       </c>
-      <c r="D29" s="8" t="inlineStr">
-        <is>
-          <t>I</t>
-        </is>
-      </c>
+      <c r="D29" s="8" t="n"/>
       <c r="E29" s="8" t="n"/>
       <c r="F29" s="8" t="n"/>
       <c r="G29" s="8" t="n"/>
@@ -5552,11 +5532,7 @@
       </c>
       <c r="D34" s="8" t="n"/>
       <c r="E34" s="8" t="n"/>
-      <c r="F34" s="8" t="inlineStr">
-        <is>
-          <t>S</t>
-        </is>
-      </c>
+      <c r="F34" s="8" t="n"/>
       <c r="G34" s="8" t="n"/>
       <c r="H34" s="8" t="n"/>
       <c r="I34" s="8" t="n"/>
@@ -7205,7 +7181,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AW51"/>
+  <dimension ref="A1:AW99"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="14.453125" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col width="6.453125" customWidth="1" style="36" min="1" max="1"/>
@@ -7880,16 +7856,8 @@
       </c>
       <c r="D13" s="8" t="n"/>
       <c r="E13" s="8" t="n"/>
-      <c r="F13" s="8" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="G13" s="8" t="inlineStr">
-        <is>
-          <t>S</t>
-        </is>
-      </c>
+      <c r="F13" s="8" t="n"/>
+      <c r="G13" s="8" t="n"/>
       <c r="H13" s="8" t="n"/>
       <c r="I13" s="8" t="n"/>
       <c r="J13" s="8" t="n"/>
@@ -7932,11 +7900,7 @@
           <t>Amora Felicya Situmrang</t>
         </is>
       </c>
-      <c r="D14" s="8" t="inlineStr">
-        <is>
-          <t>S</t>
-        </is>
-      </c>
+      <c r="D14" s="8" t="n"/>
       <c r="E14" s="8" t="n"/>
       <c r="F14" s="8" t="n"/>
       <c r="G14" s="8" t="n"/>
@@ -8028,11 +7992,7 @@
           <t>Clayton Moliver Tan</t>
         </is>
       </c>
-      <c r="D16" s="8" t="inlineStr">
-        <is>
-          <t>S</t>
-        </is>
-      </c>
+      <c r="D16" s="8" t="n"/>
       <c r="E16" s="8" t="n"/>
       <c r="F16" s="8" t="n"/>
       <c r="G16" s="8" t="n"/>
@@ -8262,11 +8222,7 @@
           <t>Kenzo Ichigo Susantio</t>
         </is>
       </c>
-      <c r="D21" s="8" t="inlineStr">
-        <is>
-          <t>S</t>
-        </is>
-      </c>
+      <c r="D21" s="8" t="n"/>
       <c r="E21" s="8" t="n"/>
       <c r="F21" s="8" t="n"/>
       <c r="G21" s="8" t="n"/>
@@ -10467,7 +10423,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AO51"/>
+  <dimension ref="A1:AW99"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="14.453125" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col width="6.453125" customWidth="1" style="36" min="1" max="1"/>
@@ -10861,17 +10817,9 @@
           <t>Celine Grace Zhang</t>
         </is>
       </c>
-      <c r="D7" s="8" t="inlineStr">
-        <is>
-          <t>S</t>
-        </is>
-      </c>
+      <c r="D7" s="8" t="n"/>
       <c r="E7" s="8" t="n"/>
-      <c r="F7" s="8" t="inlineStr">
-        <is>
-          <t>S</t>
-        </is>
-      </c>
+      <c r="F7" s="8" t="n"/>
       <c r="G7" s="8" t="n"/>
       <c r="H7" s="8" t="n"/>
       <c r="I7" s="8" t="n"/>
@@ -11287,11 +11235,7 @@
           <t>Jemia Zhevano Yamresa Kembaren</t>
         </is>
       </c>
-      <c r="D16" s="8" t="inlineStr">
-        <is>
-          <t>S</t>
-        </is>
-      </c>
+      <c r="D16" s="8" t="n"/>
       <c r="E16" s="8" t="n"/>
       <c r="F16" s="8" t="n"/>
       <c r="G16" s="8" t="n"/>
@@ -11337,11 +11281,7 @@
           <t>Jocelyn Marcella Su</t>
         </is>
       </c>
-      <c r="D17" s="8" t="inlineStr">
-        <is>
-          <t>S</t>
-        </is>
-      </c>
+      <c r="D17" s="8" t="n"/>
       <c r="E17" s="8" t="n"/>
       <c r="F17" s="8" t="n"/>
       <c r="G17" s="8" t="n"/>
@@ -11481,11 +11421,7 @@
       </c>
       <c r="D20" s="8" t="n"/>
       <c r="E20" s="8" t="n"/>
-      <c r="F20" s="8" t="inlineStr">
-        <is>
-          <t>S</t>
-        </is>
-      </c>
+      <c r="F20" s="8" t="n"/>
       <c r="G20" s="8" t="n"/>
       <c r="H20" s="8" t="n"/>
       <c r="I20" s="8" t="n"/>
@@ -11761,11 +11697,7 @@
       </c>
       <c r="D26" s="8" t="n"/>
       <c r="E26" s="8" t="n"/>
-      <c r="F26" s="8" t="inlineStr">
-        <is>
-          <t>S</t>
-        </is>
-      </c>
+      <c r="F26" s="8" t="n"/>
       <c r="G26" s="8" t="n"/>
       <c r="H26" s="8" t="n"/>
       <c r="I26" s="8" t="n"/>

</xml_diff>